<commit_message>
small changes for testing
</commit_message>
<xml_diff>
--- a/outputs/tablestat_template.xlsx
+++ b/outputs/tablestat_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\BELANDA\PhD Thesis\Code\MATLAB\amode_navigation_experiment\experiment_b\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{373B26CE-338E-419B-AB41-19D3BBCC2BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1CA7AE9-76F4-4722-9FA9-C97FFDA99F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{B592097C-7DAF-4CBB-990E-BEE084540A4C}"/>
+    <workbookView xWindow="-23136" yWindow="-96" windowWidth="23232" windowHeight="12552" activeTab="3" xr2:uid="{B592097C-7DAF-4CBB-990E-BEE084540A4C}"/>
   </bookViews>
   <sheets>
     <sheet name="kinematicEval" sheetId="1" r:id="rId1"/>
@@ -442,18 +442,6 @@
     <xf numFmtId="2" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -467,24 +455,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -503,21 +473,51 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1165,41 +1165,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17" t="s">
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17" t="s">
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
-      <c r="P1" s="17"/>
-      <c r="Q1" s="18" t="s">
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="R1" s="18"/>
-      <c r="S1" s="18"/>
-      <c r="T1" s="18"/>
-      <c r="U1" s="18"/>
-      <c r="V1" s="18" t="s">
+      <c r="R1" s="43"/>
+      <c r="S1" s="43"/>
+      <c r="T1" s="43"/>
+      <c r="U1" s="43"/>
+      <c r="V1" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="W1" s="18"/>
-      <c r="X1" s="18"/>
-      <c r="Y1" s="18"/>
-      <c r="Z1" s="18"/>
+      <c r="W1" s="43"/>
+      <c r="X1" s="43"/>
+      <c r="Y1" s="43"/>
+      <c r="Z1" s="43"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -1699,31 +1699,31 @@
       <c r="Z8" s="2"/>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17" t="s">
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17" t="s">
+      <c r="F10" s="42"/>
+      <c r="G10" s="42"/>
+      <c r="H10" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="18" t="s">
+      <c r="I10" s="42"/>
+      <c r="J10" s="42"/>
+      <c r="K10" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="L10" s="18"/>
-      <c r="M10" s="18"/>
-      <c r="N10" s="18" t="s">
+      <c r="L10" s="43"/>
+      <c r="M10" s="43"/>
+      <c r="N10" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="O10" s="18"/>
-      <c r="P10" s="18"/>
+      <c r="O10" s="43"/>
+      <c r="P10" s="43"/>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
@@ -2174,22 +2174,22 @@
       <c r="P18" s="2"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="22"/>
-      <c r="B19" s="26" t="s">
+      <c r="A19" s="18"/>
+      <c r="B19" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="27"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="26" t="s">
+      <c r="C19" s="40"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="F19" s="27"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="26" t="s">
+      <c r="F19" s="40"/>
+      <c r="G19" s="41"/>
+      <c r="H19" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="I19" s="27"/>
-      <c r="J19" s="28"/>
+      <c r="I19" s="40"/>
+      <c r="J19" s="41"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
       <c r="M19" s="3"/>
@@ -2198,32 +2198,32 @@
       <c r="P19" s="2"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="22"/>
-      <c r="B20" s="23" t="s">
+      <c r="A20" s="18"/>
+      <c r="B20" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C20" s="24" t="s">
+      <c r="C20" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="25" t="s">
+      <c r="D20" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="E20" s="23" t="s">
+      <c r="E20" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="F20" s="24" t="s">
+      <c r="F20" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="G20" s="25" t="s">
+      <c r="G20" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="H20" s="23" t="s">
+      <c r="H20" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="I20" s="24" t="s">
+      <c r="I20" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="J20" s="25" t="s">
+      <c r="J20" s="21" t="s">
         <v>13</v>
       </c>
       <c r="K20" s="2"/>
@@ -2516,95 +2516,95 @@
       <c r="P26" s="2"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A28" s="42" t="s">
+      <c r="A28" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="B28" s="29" t="s">
+      <c r="B28" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="C28" s="30"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="29" t="s">
+      <c r="C28" s="37"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="F28" s="30"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="29" t="s">
+      <c r="F28" s="37"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="I28" s="30"/>
-      <c r="J28" s="31"/>
+      <c r="I28" s="37"/>
+      <c r="J28" s="38"/>
       <c r="L28" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="43"/>
-      <c r="B29" s="39" t="s">
+      <c r="A29" s="35"/>
+      <c r="B29" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="40" t="s">
+      <c r="C29" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D29" s="41" t="s">
+      <c r="D29" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="E29" s="39" t="s">
+      <c r="E29" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="F29" s="40" t="s">
+      <c r="F29" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="G29" s="41" t="s">
+      <c r="G29" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="H29" s="39" t="s">
+      <c r="H29" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="I29" s="40" t="s">
+      <c r="I29" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="J29" s="41" t="s">
+      <c r="J29" s="31" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A30" s="32" t="s">
+      <c r="A30" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B30" s="33" t="str">
+      <c r="B30" s="23" t="str">
         <f>B12</f>
         <v>3.70 ± 1.06</v>
       </c>
-      <c r="C30" s="34" t="str">
+      <c r="C30" s="24" t="str">
         <f>E12</f>
         <v>6.71 ± 5.13</v>
       </c>
-      <c r="D30" s="35" t="str">
+      <c r="D30" s="25" t="str">
         <f>H12</f>
         <v>5.53 ± 3.92</v>
       </c>
-      <c r="E30" s="36" t="str">
+      <c r="E30" s="26" t="str">
         <f>C12</f>
         <v>3.37 ▴ 6.79</v>
       </c>
-      <c r="F30" s="37" t="str">
+      <c r="F30" s="27" t="str">
         <f>F12</f>
         <v>2.66 ▴ 17.08</v>
       </c>
-      <c r="G30" s="38" t="str">
+      <c r="G30" s="28" t="str">
         <f>I12</f>
         <v>2.96 ▴ 13.05</v>
       </c>
-      <c r="H30" s="33">
+      <c r="H30" s="23">
         <f>D12</f>
         <v>0.99600004112783203</v>
       </c>
-      <c r="I30" s="34">
+      <c r="I30" s="24">
         <f>G12</f>
         <v>0.98133763413798303</v>
       </c>
-      <c r="J30" s="35">
+      <c r="J30" s="25">
         <f>J12</f>
         <v>0.99055095826475403</v>
       </c>
@@ -2816,6 +2816,16 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="G1:K1"/>
+    <mergeCell ref="L1:P1"/>
+    <mergeCell ref="Q1:U1"/>
+    <mergeCell ref="V1:Z1"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="N10:P10"/>
     <mergeCell ref="A28:A29"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="E28:G28"/>
@@ -2823,16 +2833,6 @@
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="H19:J19"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="B1:F1"/>
-    <mergeCell ref="G1:K1"/>
-    <mergeCell ref="L1:P1"/>
-    <mergeCell ref="Q1:U1"/>
-    <mergeCell ref="V1:Z1"/>
   </mergeCells>
   <conditionalFormatting sqref="B21:D26">
     <cfRule type="expression" dxfId="34" priority="4">
@@ -2872,27 +2872,27 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17" t="s">
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17" t="s">
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="17"/>
-      <c r="P2" s="17"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
@@ -3247,27 +3247,27 @@
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17" t="s">
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="17" t="s">
+      <c r="H12" s="42"/>
+      <c r="I12" s="42"/>
+      <c r="J12" s="42"/>
+      <c r="K12" s="42"/>
+      <c r="L12" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="M12" s="17"/>
-      <c r="N12" s="17"/>
-      <c r="O12" s="17"/>
-      <c r="P12" s="17"/>
+      <c r="M12" s="42"/>
+      <c r="N12" s="42"/>
+      <c r="O12" s="42"/>
+      <c r="P12" s="42"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
@@ -3617,31 +3617,31 @@
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17" t="s">
+      <c r="C21" s="42"/>
+      <c r="D21" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17" t="s">
+      <c r="E21" s="42"/>
+      <c r="F21" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="G21" s="17"/>
+      <c r="G21" s="42"/>
       <c r="I21" s="10"/>
-      <c r="J21" s="19" t="s">
+      <c r="J21" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="K21" s="20"/>
-      <c r="L21" s="19" t="s">
+      <c r="K21" s="45"/>
+      <c r="L21" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="M21" s="20"/>
-      <c r="N21" s="19" t="s">
+      <c r="M21" s="45"/>
+      <c r="N21" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="O21" s="20"/>
+      <c r="O21" s="45"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
@@ -4019,31 +4019,31 @@
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B30" s="17" t="s">
+      <c r="B30" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17" t="s">
+      <c r="C30" s="42"/>
+      <c r="D30" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17" t="s">
+      <c r="E30" s="42"/>
+      <c r="F30" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="G30" s="17"/>
+      <c r="G30" s="42"/>
       <c r="I30" s="10"/>
-      <c r="J30" s="19" t="s">
+      <c r="J30" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="K30" s="20"/>
-      <c r="L30" s="19" t="s">
+      <c r="K30" s="45"/>
+      <c r="L30" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="M30" s="20"/>
-      <c r="N30" s="19" t="s">
+      <c r="M30" s="45"/>
+      <c r="N30" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="O30" s="20"/>
+      <c r="O30" s="45"/>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
@@ -4422,24 +4422,24 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="L30:M30"/>
+    <mergeCell ref="N30:O30"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="L2:P2"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="G12:K12"/>
+    <mergeCell ref="L12:P12"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="D21:E21"/>
     <mergeCell ref="F21:G21"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="F30:G30"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="L2:P2"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="G12:K12"/>
-    <mergeCell ref="L12:P12"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="L30:M30"/>
-    <mergeCell ref="N30:O30"/>
   </mergeCells>
   <conditionalFormatting sqref="J23:K28">
     <cfRule type="expression" dxfId="30" priority="12">
@@ -4510,27 +4510,27 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17" t="s">
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17" t="s">
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="17"/>
-      <c r="P2" s="17"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
@@ -4885,27 +4885,27 @@
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17" t="s">
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="17" t="s">
+      <c r="H12" s="42"/>
+      <c r="I12" s="42"/>
+      <c r="J12" s="42"/>
+      <c r="K12" s="42"/>
+      <c r="L12" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="M12" s="17"/>
-      <c r="N12" s="17"/>
-      <c r="O12" s="17"/>
-      <c r="P12" s="17"/>
+      <c r="M12" s="42"/>
+      <c r="N12" s="42"/>
+      <c r="O12" s="42"/>
+      <c r="P12" s="42"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
@@ -5292,18 +5292,18 @@
       <c r="P21" s="1"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17" t="s">
+      <c r="C22" s="42"/>
+      <c r="D22" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17" t="s">
+      <c r="E22" s="42"/>
+      <c r="F22" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="G22" s="17"/>
+      <c r="G22" s="42"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
@@ -5573,18 +5573,18 @@
       <c r="P31" s="1"/>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B32" s="17" t="s">
+      <c r="B32" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17" t="s">
+      <c r="C32" s="42"/>
+      <c r="D32" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17" t="s">
+      <c r="E32" s="42"/>
+      <c r="F32" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="G32" s="17"/>
+      <c r="G32" s="42"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
@@ -5817,33 +5817,33 @@
       <c r="P39" s="1"/>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B41" s="17" t="s">
+      <c r="B41" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C41" s="17"/>
-      <c r="D41" s="17" t="s">
+      <c r="C41" s="42"/>
+      <c r="D41" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17" t="s">
+      <c r="E41" s="42"/>
+      <c r="F41" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="G41" s="17"/>
-      <c r="I41" s="42" t="s">
+      <c r="G41" s="42"/>
+      <c r="I41" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="J41" s="45" t="s">
+      <c r="J41" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="K41" s="46"/>
-      <c r="L41" s="45" t="s">
+      <c r="K41" s="47"/>
+      <c r="L41" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="M41" s="46"/>
-      <c r="N41" s="45" t="s">
+      <c r="M41" s="47"/>
+      <c r="N41" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="O41" s="46"/>
+      <c r="O41" s="47"/>
     </row>
     <row r="42" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
@@ -5864,23 +5864,23 @@
       <c r="G42" t="s">
         <v>21</v>
       </c>
-      <c r="I42" s="43"/>
-      <c r="J42" s="39" t="s">
+      <c r="I42" s="35"/>
+      <c r="J42" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="K42" s="41" t="s">
+      <c r="K42" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="L42" s="39" t="s">
+      <c r="L42" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="M42" s="41" t="s">
+      <c r="M42" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="N42" s="39" t="s">
+      <c r="N42" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="O42" s="41" t="s">
+      <c r="O42" s="31" t="s">
         <v>21</v>
       </c>
     </row>
@@ -5912,30 +5912,30 @@
         <f>L14</f>
         <v>6.0778871222411297</v>
       </c>
-      <c r="I43" s="47" t="s">
+      <c r="I43" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="J43" s="44" t="str">
+      <c r="J43" s="32" t="str">
         <f t="shared" ref="J43:J48" si="0">TEXT(B4,"0.00") &amp; " ± " &amp; TEXT(C4,"0.00")</f>
         <v>3.21 ± 0.91</v>
       </c>
-      <c r="K43" s="38" t="str">
+      <c r="K43" s="28" t="str">
         <f t="shared" ref="K43:K48" si="1">TEXT(B14,"0.00") &amp; " ± " &amp; TEXT(C14,"0.00")</f>
         <v>4.09 ± 1.13</v>
       </c>
-      <c r="L43" s="44" t="str">
+      <c r="L43" s="32" t="str">
         <f t="shared" ref="L43:L48" si="2">TEXT(G4,"0.00") &amp; " ± " &amp; TEXT(H4,"0.00")</f>
         <v>6.65 ± 5.24</v>
       </c>
-      <c r="M43" s="38" t="str">
+      <c r="M43" s="28" t="str">
         <f t="shared" ref="M43:M48" si="3">TEXT(G14,"0.00") &amp; " ± " &amp; TEXT(H14,"0.00")</f>
         <v>6.07 ± 4.61</v>
       </c>
-      <c r="N43" s="44" t="str">
+      <c r="N43" s="32" t="str">
         <f t="shared" ref="N43:N48" si="4">TEXT(L4,"0.00") &amp; " ± " &amp; TEXT(M4,"0.00")</f>
         <v>5.29 ± 3.85</v>
       </c>
-      <c r="O43" s="38" t="str">
+      <c r="O43" s="28" t="str">
         <f t="shared" ref="O43:O48" si="5">TEXT(L14,"0.00") &amp; " ± " &amp; TEXT(M14,"0.00")</f>
         <v>6.08 ± 4.22</v>
       </c>
@@ -5968,7 +5968,7 @@
         <f t="shared" ref="G44:G48" si="11">L15</f>
         <v>7.0066382566082597</v>
       </c>
-      <c r="I44" s="21" t="s">
+      <c r="I44" s="17" t="s">
         <v>1</v>
       </c>
       <c r="J44" s="6" t="str">
@@ -6024,7 +6024,7 @@
         <f t="shared" si="11"/>
         <v>2.7142584235473102</v>
       </c>
-      <c r="I45" s="21" t="s">
+      <c r="I45" s="17" t="s">
         <v>2</v>
       </c>
       <c r="J45" s="6" t="str">
@@ -6080,7 +6080,7 @@
         <f t="shared" si="11"/>
         <v>1.8021812002780599</v>
       </c>
-      <c r="I46" s="21" t="s">
+      <c r="I46" s="17" t="s">
         <v>3</v>
       </c>
       <c r="J46" s="6" t="str">
@@ -6136,7 +6136,7 @@
         <f t="shared" si="11"/>
         <v>15.737257194167499</v>
       </c>
-      <c r="I47" s="21" t="s">
+      <c r="I47" s="17" t="s">
         <v>4</v>
       </c>
       <c r="J47" s="6" t="str">
@@ -6192,7 +6192,7 @@
         <f t="shared" si="11"/>
         <v>3.13020600521227</v>
       </c>
-      <c r="I48" s="21" t="s">
+      <c r="I48" s="17" t="s">
         <v>5</v>
       </c>
       <c r="J48" s="6" t="str">
@@ -6221,33 +6221,33 @@
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B50" s="17" t="s">
+      <c r="B50" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C50" s="17"/>
-      <c r="D50" s="17" t="s">
+      <c r="C50" s="42"/>
+      <c r="D50" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="E50" s="17"/>
-      <c r="F50" s="17" t="s">
+      <c r="E50" s="42"/>
+      <c r="F50" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="G50" s="17"/>
-      <c r="I50" s="42" t="s">
+      <c r="G50" s="42"/>
+      <c r="I50" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="J50" s="45" t="s">
+      <c r="J50" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="K50" s="46"/>
-      <c r="L50" s="45" t="s">
+      <c r="K50" s="47"/>
+      <c r="L50" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="M50" s="46"/>
-      <c r="N50" s="45" t="s">
+      <c r="M50" s="47"/>
+      <c r="N50" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="O50" s="46"/>
+      <c r="O50" s="47"/>
     </row>
     <row r="51" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
@@ -6268,23 +6268,23 @@
       <c r="G51" t="s">
         <v>21</v>
       </c>
-      <c r="I51" s="43"/>
-      <c r="J51" s="39" t="s">
+      <c r="I51" s="35"/>
+      <c r="J51" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="K51" s="41" t="s">
+      <c r="K51" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="L51" s="39" t="s">
+      <c r="L51" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="M51" s="41" t="s">
+      <c r="M51" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="N51" s="39" t="s">
+      <c r="N51" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="O51" s="41" t="s">
+      <c r="O51" s="31" t="s">
         <v>21</v>
       </c>
     </row>
@@ -6316,30 +6316,30 @@
         <f>N14</f>
         <v>3.6630578537298102</v>
       </c>
-      <c r="I52" s="47" t="s">
+      <c r="I52" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="J52" s="44" t="str">
+      <c r="J52" s="32" t="str">
         <f t="shared" ref="J52:J57" si="12">TEXT(D4,"0.00") &amp; " ▴ " &amp; TEXT(E4,"0.00")</f>
         <v>2.87 ▴ 5.27</v>
       </c>
-      <c r="K52" s="38" t="str">
+      <c r="K52" s="28" t="str">
         <f t="shared" ref="K52:K57" si="13">TEXT(D14,"0.00") &amp; " ▴ " &amp; TEXT(E14,"0.00")</f>
         <v>3.87 ▴ 6.81</v>
       </c>
-      <c r="L52" s="44" t="str">
+      <c r="L52" s="32" t="str">
         <f t="shared" ref="L52:L57" si="14">TEXT(I4,"0.00") &amp; " ▴ " &amp; TEXT(J4,"0.00")</f>
         <v>1.67 ▴ 17.07</v>
       </c>
-      <c r="M52" s="38" t="str">
+      <c r="M52" s="28" t="str">
         <f t="shared" ref="M52:M57" si="15">TEXT(I14,"0.00") &amp; " ▴ " &amp; TEXT(J14,"0.00")</f>
         <v>2.86 ▴ 14.53</v>
       </c>
-      <c r="N52" s="44" t="str">
+      <c r="N52" s="32" t="str">
         <f t="shared" ref="N52:N57" si="16">TEXT(N4,"0.00") &amp; " ▴ " &amp; TEXT(O4,"0.00")</f>
         <v>2.39 ▴ 13.05</v>
       </c>
-      <c r="O52" s="38" t="str">
+      <c r="O52" s="28" t="str">
         <f t="shared" ref="O52:O57" si="17">TEXT(N14,"0.00") &amp; " ▴ " &amp; TEXT(O14,"0.00")</f>
         <v>3.66 ▴ 11.92</v>
       </c>
@@ -6372,7 +6372,7 @@
         <f t="shared" ref="G53:G57" si="23">N15</f>
         <v>6.6377020590646802</v>
       </c>
-      <c r="I53" s="21" t="s">
+      <c r="I53" s="17" t="s">
         <v>1</v>
       </c>
       <c r="J53" s="6" t="str">
@@ -6428,7 +6428,7 @@
         <f t="shared" si="23"/>
         <v>2.6486084869154398</v>
       </c>
-      <c r="I54" s="21" t="s">
+      <c r="I54" s="17" t="s">
         <v>2</v>
       </c>
       <c r="J54" s="6" t="str">
@@ -6484,7 +6484,7 @@
         <f t="shared" si="23"/>
         <v>1.8032077594970399</v>
       </c>
-      <c r="I55" s="21" t="s">
+      <c r="I55" s="17" t="s">
         <v>3</v>
       </c>
       <c r="J55" s="6" t="str">
@@ -6540,7 +6540,7 @@
         <f t="shared" si="23"/>
         <v>16.4508394030658</v>
       </c>
-      <c r="I56" s="21" t="s">
+      <c r="I56" s="17" t="s">
         <v>4</v>
       </c>
       <c r="J56" s="6" t="str">
@@ -6596,7 +6596,7 @@
         <f t="shared" si="23"/>
         <v>3.1473137309992398</v>
       </c>
-      <c r="I57" s="21" t="s">
+      <c r="I57" s="17" t="s">
         <v>5</v>
       </c>
       <c r="J57" s="6" t="str">
@@ -6626,12 +6626,12 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="L2:P2"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="G12:K12"/>
+    <mergeCell ref="L12:P12"/>
     <mergeCell ref="N50:O50"/>
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="D41:E41"/>
@@ -6646,12 +6646,12 @@
     <mergeCell ref="L50:M50"/>
     <mergeCell ref="I41:I42"/>
     <mergeCell ref="I50:I51"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="L2:P2"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="G12:K12"/>
-    <mergeCell ref="L12:P12"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F32:G32"/>
   </mergeCells>
   <conditionalFormatting sqref="J43:K48">
     <cfRule type="expression" dxfId="18" priority="100" stopIfTrue="1">
@@ -6733,24 +6733,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17" t="s">
+      <c r="C1" s="42"/>
+      <c r="D1" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17" t="s">
+      <c r="E1" s="42"/>
+      <c r="F1" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17" t="s">
+      <c r="G1" s="42"/>
+      <c r="H1" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B2" t="s">

</xml_diff>